<commit_message>
Clean docs, harden deeplink login prep
</commit_message>
<xml_diff>
--- a/testcases/deeplinks/DeeplinkTestCases.xlsx
+++ b/testcases/deeplinks/DeeplinkTestCases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marnisaisanjay/Documents/personalprojects/AppPilot/testcases/deeplinks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A52388D-FCD1-4445-B66B-21819CD21E7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D654B7FF-8551-E644-B05A-D335056C810E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{C5943666-9D12-0C47-8784-2B49B0DE6ECC}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="49">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -187,78 +187,6 @@
   </si>
   <si>
     <t>Researcher screen with prompt "Help me prepare to address ’s concerns. Summarize their recent issues, escalation history, usage patterns, business priorities, and any relevant industry or market context. Deliver a 3-page brief with their top concerns and how we’re addressing them, including talking points and objection handing." or Message saying researcher is not available</t>
-  </si>
-  <si>
-    <t>TC025</t>
-  </si>
-  <si>
-    <t>TC026</t>
-  </si>
-  <si>
-    <t>TC027</t>
-  </si>
-  <si>
-    <t>TC028</t>
-  </si>
-  <si>
-    <t>TC029</t>
-  </si>
-  <si>
-    <t>TC030</t>
-  </si>
-  <si>
-    <t>TC031</t>
-  </si>
-  <si>
-    <t>TC032</t>
-  </si>
-  <si>
-    <t>TC033</t>
-  </si>
-  <si>
-    <t>TC034</t>
-  </si>
-  <si>
-    <t>TC035</t>
-  </si>
-  <si>
-    <t>TC036</t>
-  </si>
-  <si>
-    <t>TC037</t>
-  </si>
-  <si>
-    <t>TC038</t>
-  </si>
-  <si>
-    <t>TC039</t>
-  </si>
-  <si>
-    <t>TC040</t>
-  </si>
-  <si>
-    <t>TC041</t>
-  </si>
-  <si>
-    <t>TC042</t>
-  </si>
-  <si>
-    <t>TC043</t>
-  </si>
-  <si>
-    <t>TC044</t>
-  </si>
-  <si>
-    <t>TC045</t>
-  </si>
-  <si>
-    <t>TC046</t>
-  </si>
-  <si>
-    <t>TC047</t>
-  </si>
-  <si>
-    <t>TC048</t>
   </si>
 </sst>
 </file>
@@ -715,10 +643,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1814,21 +1738,11 @@
       </c>
     </row>
     <row r="27" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>8</v>
-      </c>
+      <c r="A27" s="12"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="9"/>
       <c r="F27" s="11"/>
       <c r="G27" s="11"/>
       <c r="H27" s="11"/>
@@ -1852,21 +1766,11 @@
       <c r="Z27" s="11"/>
     </row>
     <row r="28" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>8</v>
-      </c>
+      <c r="A28" s="13"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="11"/>
       <c r="G28" s="11"/>
       <c r="H28" s="11"/>
@@ -1890,21 +1794,11 @@
       <c r="Z28" s="11"/>
     </row>
     <row r="29" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D29" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="E29" s="9" t="s">
-        <v>8</v>
-      </c>
+      <c r="A29" s="12"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="9"/>
       <c r="F29" s="11"/>
       <c r="G29" s="11"/>
       <c r="H29" s="11"/>
@@ -1928,21 +1822,11 @@
       <c r="Z29" s="11"/>
     </row>
     <row r="30" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E30" s="7" t="s">
-        <v>8</v>
-      </c>
+      <c r="A30" s="13"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="7"/>
       <c r="F30" s="11"/>
       <c r="G30" s="11"/>
       <c r="H30" s="11"/>
@@ -1966,72 +1850,32 @@
       <c r="Z30" s="11"/>
     </row>
     <row r="31" spans="1:26" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E31" s="9" t="s">
-        <v>8</v>
-      </c>
+      <c r="A31" s="12"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="9"/>
     </row>
     <row r="32" spans="1:26" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E32" s="7" t="s">
-        <v>8</v>
-      </c>
+      <c r="A32" s="13"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="7"/>
     </row>
     <row r="33" spans="1:26" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="E33" s="9" t="s">
-        <v>8</v>
-      </c>
+      <c r="A33" s="12"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="9"/>
     </row>
     <row r="34" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E34" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A34" s="13"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="7"/>
       <c r="F34" s="11"/>
       <c r="G34" s="11"/>
       <c r="H34" s="11"/>
@@ -2055,21 +1899,11 @@
       <c r="Z34" s="11"/>
     </row>
     <row r="35" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>11</v>
-      </c>
+      <c r="A35" s="12"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="9"/>
       <c r="F35" s="11"/>
       <c r="G35" s="11"/>
       <c r="H35" s="11"/>
@@ -2093,21 +1927,11 @@
       <c r="Z35" s="11"/>
     </row>
     <row r="36" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D36" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E36" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A36" s="13"/>
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="7"/>
       <c r="F36" s="11"/>
       <c r="G36" s="11"/>
       <c r="H36" s="11"/>
@@ -2131,21 +1955,11 @@
       <c r="Z36" s="11"/>
     </row>
     <row r="37" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C37" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="E37" s="9" t="s">
-        <v>11</v>
-      </c>
+      <c r="A37" s="12"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="9"/>
       <c r="F37" s="11"/>
       <c r="G37" s="11"/>
       <c r="H37" s="11"/>
@@ -2169,72 +1983,32 @@
       <c r="Z37" s="11"/>
     </row>
     <row r="38" spans="1:26" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D38" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E38" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A38" s="13"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="7"/>
     </row>
     <row r="39" spans="1:26" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="B39" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C39" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E39" s="9" t="s">
-        <v>11</v>
-      </c>
+      <c r="A39" s="12"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="9"/>
     </row>
     <row r="40" spans="1:26" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D40" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E40" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A40" s="13"/>
+      <c r="B40" s="6"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="7"/>
     </row>
     <row r="41" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D41" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E41" s="9" t="s">
-        <v>8</v>
-      </c>
+      <c r="A41" s="12"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="9"/>
       <c r="F41" s="11"/>
       <c r="G41" s="11"/>
       <c r="H41" s="11"/>
@@ -2258,21 +2032,11 @@
       <c r="Z41" s="11"/>
     </row>
     <row r="42" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C42" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D42" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E42" s="7" t="s">
-        <v>8</v>
-      </c>
+      <c r="A42" s="13"/>
+      <c r="B42" s="6"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="7"/>
       <c r="F42" s="11"/>
       <c r="G42" s="11"/>
       <c r="H42" s="11"/>
@@ -2296,21 +2060,11 @@
       <c r="Z42" s="11"/>
     </row>
     <row r="43" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C43" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="E43" s="9" t="s">
-        <v>8</v>
-      </c>
+      <c r="A43" s="12"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="9"/>
       <c r="F43" s="11"/>
       <c r="G43" s="11"/>
       <c r="H43" s="11"/>
@@ -2334,55 +2088,25 @@
       <c r="Z43" s="11"/>
     </row>
     <row r="44" spans="1:26" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C44" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E44" s="7" t="s">
-        <v>8</v>
-      </c>
+      <c r="A44" s="13"/>
+      <c r="B44" s="6"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="7"/>
     </row>
     <row r="45" spans="1:26" ht="142" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C45" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="E45" s="9" t="s">
-        <v>8</v>
-      </c>
+      <c r="A45" s="12"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="9"/>
     </row>
     <row r="46" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="B46" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C46" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D46" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E46" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A46" s="13"/>
+      <c r="B46" s="6"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="7"/>
       <c r="F46" s="11"/>
       <c r="G46" s="11"/>
       <c r="H46" s="11"/>
@@ -2406,21 +2130,11 @@
       <c r="Z46" s="11"/>
     </row>
     <row r="47" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="B47" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C47" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D47" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E47" s="9" t="s">
-        <v>11</v>
-      </c>
+      <c r="A47" s="12"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="9"/>
       <c r="F47" s="11"/>
       <c r="G47" s="11"/>
       <c r="H47" s="11"/>
@@ -2444,21 +2158,11 @@
       <c r="Z47" s="11"/>
     </row>
     <row r="48" spans="1:26" s="2" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C48" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E48" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A48" s="13"/>
+      <c r="B48" s="6"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="6"/>
+      <c r="E48" s="7"/>
       <c r="F48" s="11"/>
       <c r="G48" s="11"/>
       <c r="H48" s="11"/>
@@ -2482,38 +2186,18 @@
       <c r="Z48" s="11"/>
     </row>
     <row r="49" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="B49" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C49" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E49" s="9" t="s">
-        <v>11</v>
-      </c>
+      <c r="A49" s="12"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="6"/>
+      <c r="E49" s="9"/>
     </row>
     <row r="50" spans="1:5" ht="144" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="B50" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C50" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="E50" s="7" t="s">
-        <v>11</v>
-      </c>
+      <c r="A50" s="13"/>
+      <c r="B50" s="6"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2524,15 +2208,11 @@
     <hyperlink ref="B3" r:id="rId2" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{FB00C298-129B-074E-9E51-BE087D0993EF}"/>
     <hyperlink ref="B22" r:id="rId3" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{1E88FB97-6BD6-2447-80B5-13A07BC875EE}"/>
     <hyperlink ref="B17" r:id="rId4" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{FB67E84E-3C8F-EF43-9A44-269EA3D1B808}"/>
-    <hyperlink ref="B34" r:id="rId5" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{C850BD82-41A7-D440-9EFD-1B26CBE86880}"/>
-    <hyperlink ref="B27" r:id="rId6" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{8DC9D010-9A9F-4643-9F91-E9E4EC729473}"/>
-    <hyperlink ref="B46" r:id="rId7" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{66FEF975-C2B6-C64D-9913-E3D368E31245}"/>
-    <hyperlink ref="B41" r:id="rId8" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{C537088B-A9C6-0A45-9C4B-39838C643DDE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
-    <tablePart r:id="rId9"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>